<commit_message>
feat(release-note): tô màu dropdown ステータス trong template xlsx
Conditional formatting trên đúng vùng dropdown Status (E20:E27 E30:E36 E39:E48 E50:E56):
Open xám · In Progress vàng · Done xanh lá · No Need xanh nhạt.
</commit_message>
<xml_diff>
--- a/skills/release-note/assets/release-note-template.xlsx
+++ b/skills/release-note/assets/release-note-template.xlsx
@@ -1308,7 +1308,7 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1498,6 +1498,54 @@
           <color theme="4" tint="0.399975585192419"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="003C3C3C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E6E6E6"/>
+          <bgColor rgb="00E6E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="005C4A00"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFE599"/>
+          <bgColor rgb="00FFE599"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001E4D1E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00B6D7A8"/>
+          <bgColor rgb="00B6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="002E4E6B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00CFE2F3"/>
+          <bgColor rgb="00CFE2F3"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
@@ -1907,7 +1955,11 @@
         </is>
       </c>
       <c r="B4" s="80" t="n"/>
-      <c r="C4" s="83" t="n"/>
+      <c r="C4" s="83" t="inlineStr">
+        <is>
+          <t>https://stg.co-medical.mynavi.jp/</t>
+        </is>
+      </c>
       <c r="D4" s="82" t="n"/>
       <c r="E4" s="82" t="n"/>
       <c r="F4" s="80" t="n"/>
@@ -2280,7 +2332,11 @@
     <row r="16" ht="105" customHeight="1">
       <c r="A16" s="38" t="n"/>
       <c r="B16" s="39" t="n"/>
-      <c r="C16" s="40" t="n"/>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>https://mynavi-sys.backlog.com/view/MAG_UNEI-14532</t>
+        </is>
+      </c>
       <c r="D16" s="41" t="n"/>
       <c r="E16" s="42" t="n"/>
       <c r="F16" s="42" t="n"/>
@@ -2765,7 +2821,11 @@
     </row>
     <row r="36" ht="95.25" customHeight="1">
       <c r="A36" s="60" t="n"/>
-      <c r="B36" s="62" t="n"/>
+      <c r="B36" s="62" t="inlineStr">
+        <is>
+          <t>https://github.com/mynavi-group/co-medical/pull/3017</t>
+        </is>
+      </c>
       <c r="C36" s="55" t="n"/>
       <c r="D36" s="52" t="n"/>
       <c r="E36" s="53" t="n"/>
@@ -2836,7 +2896,11 @@
       <c r="C39" s="65" t="n"/>
       <c r="D39" s="52" t="n"/>
       <c r="E39" s="53" t="n"/>
-      <c r="F39" s="66" t="n"/>
+      <c r="F39" s="66" t="inlineStr">
+        <is>
+          <t>https://github.com/mynavi-group/co-medical/actions/runs/35970019675/</t>
+        </is>
+      </c>
       <c r="G39" s="21" t="n"/>
       <c r="H39" s="21" t="n"/>
       <c r="I39" s="21" t="n"/>
@@ -2941,7 +3005,11 @@
       <c r="C44" s="65" t="n"/>
       <c r="D44" s="52" t="n"/>
       <c r="E44" s="53" t="n"/>
-      <c r="F44" s="62" t="n"/>
+      <c r="F44" s="62" t="inlineStr">
+        <is>
+          <t>https://stg.co-medical.mynavi.jp/search/search.php</t>
+        </is>
+      </c>
       <c r="G44" s="21" t="n"/>
       <c r="H44" s="21" t="n"/>
       <c r="I44" s="21" t="n"/>
@@ -3252,6 +3320,20 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
+  <conditionalFormatting sqref="E20:E27 E30:E36 E39:E48 E50:E56">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="17">
+      <formula>"Open"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="18">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="19">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="20">
+      <formula>"No Need"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="N12:O12 N15:O18 Q16:R26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Testing,OK,Re-open,Not Test"</formula1>

</xml_diff>

<commit_message>
fix(release-note): clean leftover co-medical sample content from xlsx template (C4, C16, B36, F39, F44 incl. hyperlinks)
</commit_message>
<xml_diff>
--- a/skills/release-note/assets/release-note-template.xlsx
+++ b/skills/release-note/assets/release-note-template.xlsx
@@ -1955,11 +1955,7 @@
         </is>
       </c>
       <c r="B4" s="80" t="n"/>
-      <c r="C4" s="83" t="inlineStr">
-        <is>
-          <t>https://stg.co-medical.mynavi.jp/</t>
-        </is>
-      </c>
+      <c r="C4" s="83" t="inlineStr"/>
       <c r="D4" s="82" t="n"/>
       <c r="E4" s="82" t="n"/>
       <c r="F4" s="80" t="n"/>
@@ -2332,11 +2328,7 @@
     <row r="16" ht="105" customHeight="1">
       <c r="A16" s="38" t="n"/>
       <c r="B16" s="39" t="n"/>
-      <c r="C16" s="40" t="inlineStr">
-        <is>
-          <t>https://mynavi-sys.backlog.com/view/MAG_UNEI-14532</t>
-        </is>
-      </c>
+      <c r="C16" s="40" t="inlineStr"/>
       <c r="D16" s="41" t="n"/>
       <c r="E16" s="42" t="n"/>
       <c r="F16" s="42" t="n"/>
@@ -2821,11 +2813,7 @@
     </row>
     <row r="36" ht="95.25" customHeight="1">
       <c r="A36" s="60" t="n"/>
-      <c r="B36" s="62" t="inlineStr">
-        <is>
-          <t>https://github.com/mynavi-group/co-medical/pull/3017</t>
-        </is>
-      </c>
+      <c r="B36" s="62" t="inlineStr"/>
       <c r="C36" s="55" t="n"/>
       <c r="D36" s="52" t="n"/>
       <c r="E36" s="53" t="n"/>
@@ -2896,11 +2884,7 @@
       <c r="C39" s="65" t="n"/>
       <c r="D39" s="52" t="n"/>
       <c r="E39" s="53" t="n"/>
-      <c r="F39" s="66" t="inlineStr">
-        <is>
-          <t>https://github.com/mynavi-group/co-medical/actions/runs/35970019675/</t>
-        </is>
-      </c>
+      <c r="F39" s="66" t="inlineStr"/>
       <c r="G39" s="21" t="n"/>
       <c r="H39" s="21" t="n"/>
       <c r="I39" s="21" t="n"/>
@@ -3005,11 +2989,7 @@
       <c r="C44" s="65" t="n"/>
       <c r="D44" s="52" t="n"/>
       <c r="E44" s="53" t="n"/>
-      <c r="F44" s="62" t="inlineStr">
-        <is>
-          <t>https://stg.co-medical.mynavi.jp/search/search.php</t>
-        </is>
-      </c>
+      <c r="F44" s="62" t="inlineStr"/>
       <c r="G44" s="21" t="n"/>
       <c r="H44" s="21" t="n"/>
       <c r="I44" s="21" t="n"/>
@@ -3342,13 +3322,6 @@
       <formula1>"Open,In Progress,Done,No Need"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" display="https://stg.co-medical.mynavi.jp/" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" display="MAG_UNEI-14532 【マイナビコメディカル】Github Actionsの再構築" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" display="Merge PR #3017&#10;ーーーー&#10;PR #3017 マージ" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" display="https://github.com/mynavi-group/co-medical/actions/runs/35970019675/" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" display="https://stg.co-medical.mynavi.jp/&#10;https://stg.co-medical.mynavi.jp/search/&#10;https://stg.co-medical.mynavi.jp/search/search.php&#10;https://stg.co-medical.mynavi.jp/search/30300140/ar/st/1001,1002,1003,1004,1011,1008/&#10;https://stg.co-medical.mynavi.jp/contents/" r:id="rId5"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>